<commit_message>
Add AI decision confidence to planning results
</commit_message>
<xml_diff>
--- a/data/raw/SIH26027_Stage_B1_Starter_Dataset.xlsx
+++ b/data/raw/SIH26027_Stage_B1_Starter_Dataset.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J11"/>
+  <dimension ref="A1:J26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -486,7 +486,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>M001</t>
+          <t>M101</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -536,7 +536,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>M002</t>
+          <t>M102</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -586,31 +586,31 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>M003</t>
+          <t>M103</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>Traction Distribution</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>OHE</t>
+          <t>Track</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>SEC-B</t>
+          <t>SEC-A</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>OHE inspection</t>
+          <t>Rail joint repair</t>
         </is>
       </c>
       <c r="F4" t="n">
-        <v>2</v>
+        <v>1.5</v>
       </c>
       <c r="G4" t="inlineStr">
         <is>
@@ -619,12 +619,12 @@
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>OHE Block</t>
+          <t>Track Block</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -636,27 +636,27 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>M004</t>
+          <t>M104</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>Traction Distribution</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>Track</t>
+          <t>OHE</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>SEC-C</t>
+          <t>SEC-A</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Rail joint repair</t>
+          <t>OHE component inspection</t>
         </is>
       </c>
       <c r="F5" t="n">
@@ -664,17 +664,17 @@
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>Track Block</t>
+          <t>OHE Block</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -686,40 +686,40 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>M005</t>
+          <t>M105</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Signal &amp; Telecom</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Signal</t>
+          <t>Track</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>SEC-C</t>
+          <t>SEC-B</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Signal testing</t>
+          <t>Track geometry inspection</t>
         </is>
       </c>
       <c r="F6" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Medium</t>
+          <t>High</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
@@ -736,45 +736,45 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>M006</t>
+          <t>M106</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>Traction Distribution</t>
+          <t>Signal &amp; Telecom</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>OHE</t>
+          <t>Signal</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>SEC-A</t>
+          <t>SEC-B</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>OHE component inspection</t>
+          <t>Interlocking equipment check</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>1.5</v>
+        <v>1</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Low</t>
+          <t>High</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>OHE Block</t>
+          <t>Track Block</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -786,17 +786,17 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>M007</t>
+          <t>M107</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Engineering</t>
+          <t>Traction Distribution</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>Track</t>
+          <t>OHE</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -806,7 +806,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Track geometry inspection</t>
+          <t>OHE inspection</t>
         </is>
       </c>
       <c r="F8" t="n">
@@ -819,12 +819,12 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>Track Block</t>
+          <t>OHE Block</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -836,17 +836,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>M008</t>
+          <t>M108</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Signal &amp; Telecom</t>
+          <t>Engineering</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>Signal</t>
+          <t>Track</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -856,7 +856,7 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>Interlocking equipment check</t>
+          <t>Sleeper replacement</t>
         </is>
       </c>
       <c r="F9" t="n">
@@ -864,12 +864,12 @@
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>High</t>
+          <t>Low</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
@@ -886,7 +886,7 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>M009</t>
+          <t>M109</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
@@ -896,21 +896,21 @@
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>Bridge</t>
+          <t>Track</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
         <is>
-          <t>SEC-D</t>
+          <t>SEC-C</t>
         </is>
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Bridge structural inspection</t>
+          <t>Rail inspection</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -919,7 +919,7 @@
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
@@ -936,48 +936,798 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>M010</t>
+          <t>M110</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
+          <t>Signal &amp; Telecom</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>Signal</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>SEC-C</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Signal testing</t>
+        </is>
+      </c>
+      <c r="F11" t="n">
+        <v>1</v>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H11" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="I11" t="inlineStr">
+        <is>
+          <t>Track Block</t>
+        </is>
+      </c>
+      <c r="J11" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>M111</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>Track</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>SEC-C</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Rail joint repair</t>
+        </is>
+      </c>
+      <c r="F12" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H12" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="I12" t="inlineStr">
+        <is>
+          <t>Track Block</t>
+        </is>
+      </c>
+      <c r="J12" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>M112</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
           <t>Traction Distribution</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C13" t="inlineStr">
         <is>
           <t>OHE</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>SEC-C</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>OHE wire inspection</t>
+        </is>
+      </c>
+      <c r="F13" t="n">
+        <v>2</v>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H13" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="I13" t="inlineStr">
+        <is>
+          <t>OHE Block</t>
+        </is>
+      </c>
+      <c r="J13" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>M113</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>Bridge</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
         <is>
           <t>SEC-D</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Bridge structural inspection</t>
+        </is>
+      </c>
+      <c r="F14" t="n">
+        <v>3</v>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H14" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="I14" t="inlineStr">
+        <is>
+          <t>Track Block</t>
+        </is>
+      </c>
+      <c r="J14" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>M114</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>Traction Distribution</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>OHE</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>SEC-D</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
         <is>
           <t>OHE wire inspection</t>
         </is>
       </c>
-      <c r="F11" t="n">
+      <c r="F15" t="n">
         <v>2</v>
       </c>
-      <c r="G11" t="inlineStr">
+      <c r="G15" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="H11" t="inlineStr">
+      <c r="H15" t="inlineStr">
         <is>
           <t>2026-09-14</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr">
+      <c r="I15" t="inlineStr">
         <is>
           <t>OHE Block</t>
         </is>
       </c>
-      <c r="J11" t="inlineStr">
+      <c r="J15" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>M115</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Signal &amp; Telecom</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>Signal</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>SEC-D</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Signal equipment testing</t>
+        </is>
+      </c>
+      <c r="F16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H16" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="I16" t="inlineStr">
+        <is>
+          <t>Track Block</t>
+        </is>
+      </c>
+      <c r="J16" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>M116</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>Track</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>SEC-D</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Track alignment check</t>
+        </is>
+      </c>
+      <c r="F17" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H17" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="I17" t="inlineStr">
+        <is>
+          <t>Track Block</t>
+        </is>
+      </c>
+      <c r="J17" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>M117</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>Track</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>SEC-E</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Rail inspection</t>
+        </is>
+      </c>
+      <c r="F18" t="n">
+        <v>2</v>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H18" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="I18" t="inlineStr">
+        <is>
+          <t>Track Block</t>
+        </is>
+      </c>
+      <c r="J18" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>M118</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Signal &amp; Telecom</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>Signal</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>SEC-E</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Signal maintenance</t>
+        </is>
+      </c>
+      <c r="F19" t="n">
+        <v>1</v>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H19" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+      <c r="I19" t="inlineStr">
+        <is>
+          <t>Track Block</t>
+        </is>
+      </c>
+      <c r="J19" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>M119</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>Traction Distribution</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>OHE</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>SEC-E</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>OHE inspection</t>
+        </is>
+      </c>
+      <c r="F20" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H20" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+      <c r="I20" t="inlineStr">
+        <is>
+          <t>OHE Block</t>
+        </is>
+      </c>
+      <c r="J20" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>M120</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>Track</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>SEC-F</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Track geometry inspection</t>
+        </is>
+      </c>
+      <c r="F21" t="n">
+        <v>2</v>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H21" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+      <c r="I21" t="inlineStr">
+        <is>
+          <t>Track Block</t>
+        </is>
+      </c>
+      <c r="J21" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>M121</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>Signal &amp; Telecom</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>Signal</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>SEC-F</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Signal testing</t>
+        </is>
+      </c>
+      <c r="F22" t="n">
+        <v>1</v>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>Low</t>
+        </is>
+      </c>
+      <c r="H22" t="inlineStr">
+        <is>
+          <t>2026-09-22</t>
+        </is>
+      </c>
+      <c r="I22" t="inlineStr">
+        <is>
+          <t>Track Block</t>
+        </is>
+      </c>
+      <c r="J22" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>M122</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>Traction Distribution</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>OHE</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>SEC-F</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>OHE component inspection</t>
+        </is>
+      </c>
+      <c r="F23" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H23" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
+        </is>
+      </c>
+      <c r="I23" t="inlineStr">
+        <is>
+          <t>OHE Block</t>
+        </is>
+      </c>
+      <c r="J23" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>M123</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>Track</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>SEC-G</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Rail joint repair</t>
+        </is>
+      </c>
+      <c r="F24" t="n">
+        <v>1</v>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>Track Block</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>M124</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>Engineering</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>Track</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>SEC-G</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Track inspection</t>
+        </is>
+      </c>
+      <c r="F25" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>2026-09-23</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>Track Block</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>M125</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>Signal &amp; Telecom</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>Signal</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>SEC-G</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Interlocking test</t>
+        </is>
+      </c>
+      <c r="F26" t="n">
+        <v>1</v>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>2026-09-17</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Track Block</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
         <is>
           <t>Open</t>
         </is>
@@ -994,7 +1744,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E9"/>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1027,7 +1777,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>T101</t>
+          <t>T201</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1037,12 +1787,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>08:30</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>09:45</t>
+          <t>08:45</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -1054,7 +1804,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>T102</t>
+          <t>T202</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1064,12 +1814,12 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>10:15</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>11:15</t>
+          <t>10:30</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -1081,7 +1831,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>T103</t>
+          <t>T203</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1091,12 +1841,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>13:45</t>
+          <t>12:15</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -1108,34 +1858,34 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>T104</t>
+          <t>T204</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>SEC-B</t>
+          <t>SEC-A</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>10:15</t>
+          <t>15:20</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Passenger</t>
+          <t>Express</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>T105</t>
+          <t>T205</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1145,96 +1895,690 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>08:45</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>12:45</t>
+          <t>09:00</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Passenger</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>T106</t>
+          <t>T206</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>SEC-C</t>
+          <t>SEC-B</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>09:00</t>
+          <t>10:30</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>09:15</t>
+          <t>10:50</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Passenger</t>
+          <t>Express</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>T107</t>
+          <t>T207</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>SEC-C</t>
+          <t>SEC-B</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>12:15</t>
+          <t>12:45</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Express</t>
+          <t>Passenger</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>T108</t>
+          <t>T208</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
+          <t>SEC-B</t>
+        </is>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>15:15</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Express</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
+          <t>T209</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>SEC-C</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>Passenger</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>T210</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>SEC-C</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>11:20</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>Express</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>T211</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>SEC-C</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>Express</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>T212</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>SEC-C</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>Passenger</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>T213</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
           <t>SEC-D</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>09:45</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Express</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>T214</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>SEC-D</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>Passenger</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>T215</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>SEC-D</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
         <is>
           <t>14:00</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>14:15</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>14:20</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>Express</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>T216</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>SEC-D</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>16:45</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>Passenger</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>T217</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>SEC-E</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>08:30</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>08:45</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Passenger</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>T218</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>SEC-E</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>10:45</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Express</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr">
+        <is>
+          <t>T219</t>
+        </is>
+      </c>
+      <c r="B20" t="inlineStr">
+        <is>
+          <t>SEC-E</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="D20" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Passenger</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" t="inlineStr">
+        <is>
+          <t>T220</t>
+        </is>
+      </c>
+      <c r="B21" t="inlineStr">
+        <is>
+          <t>SEC-E</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
+          <t>15:45</t>
+        </is>
+      </c>
+      <c r="D21" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>Express</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" t="inlineStr">
+        <is>
+          <t>T221</t>
+        </is>
+      </c>
+      <c r="B22" t="inlineStr">
+        <is>
+          <t>SEC-F</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>09:15</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>Express</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" t="inlineStr">
+        <is>
+          <t>T222</t>
+        </is>
+      </c>
+      <c r="B23" t="inlineStr">
+        <is>
+          <t>SEC-F</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="D23" t="inlineStr">
+        <is>
+          <t>11:45</t>
+        </is>
+      </c>
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Passenger</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" t="inlineStr">
+        <is>
+          <t>T223</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>SEC-F</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>13:45</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>14:00</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Express</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>T224</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>SEC-F</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>16:15</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Passenger</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>T225</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>SEC-G</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>08:15</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>08:30</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Passenger</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>T226</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>SEC-G</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Express</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>T227</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>SEC-G</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Passenger</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>T228</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>SEC-G</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>14:45</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Express</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>T229</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>SEC-A</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>16:45</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Passenger</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>T230</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>SEC-D</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>13:15</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
         <is>
           <t>Express</t>
         </is>
@@ -1251,7 +2595,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G10"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1294,7 +2638,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>B001</t>
+          <t>B101</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1304,12 +2648,12 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="D2" t="inlineStr">
+        <is>
           <t>10:00</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>11:00</t>
         </is>
       </c>
       <c r="E2" t="n">
@@ -1329,7 +2673,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>B002</t>
+          <t>B102</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1339,16 +2683,16 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>10:45</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>13:30</t>
+          <t>12:00</t>
         </is>
       </c>
       <c r="E3" t="n">
-        <v>2</v>
+        <v>1.25</v>
       </c>
       <c r="F3" t="inlineStr">
         <is>
@@ -1364,7 +2708,7 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>B003</t>
+          <t>B103</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
@@ -1374,12 +2718,12 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>12:30</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>16:00</t>
+          <t>14:30</t>
         </is>
       </c>
       <c r="E4" t="n">
@@ -1399,30 +2743,30 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>B004</t>
+          <t>B104</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>SEC-B</t>
+          <t>SEC-A</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>15:30</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>17:30</t>
         </is>
       </c>
       <c r="E5" t="n">
-        <v>1.5</v>
+        <v>2</v>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>OHE Block</t>
+          <t>Track Block</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
@@ -1434,7 +2778,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>B005</t>
+          <t>B105</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
@@ -1444,12 +2788,12 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>09:15</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>11:15</t>
         </is>
       </c>
       <c r="E6" t="n">
@@ -1469,22 +2813,22 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>B006</t>
+          <t>B106</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>SEC-C</t>
+          <t>SEC-B</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>09:30</t>
+          <t>11:00</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>11:30</t>
+          <t>13:00</t>
         </is>
       </c>
       <c r="E7" t="n">
@@ -1492,7 +2836,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>Track Block</t>
+          <t>OHE Block</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
@@ -1504,22 +2848,22 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>B007</t>
+          <t>B107</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>SEC-C</t>
+          <t>SEC-B</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>12:30</t>
+          <t>13:30</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>14:00</t>
+          <t>15:00</t>
         </is>
       </c>
       <c r="E8" t="n">
@@ -1539,26 +2883,26 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>B008</t>
+          <t>B108</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>SEC-D</t>
+          <t>SEC-B</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>15:45</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>13:00</t>
+          <t>17:45</t>
         </is>
       </c>
       <c r="E9" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F9" t="inlineStr">
         <is>
@@ -1574,33 +2918,348 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>B009</t>
+          <t>B109</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
+          <t>SEC-C</t>
+        </is>
+      </c>
+      <c r="C10" t="inlineStr">
+        <is>
+          <t>09:30</t>
+        </is>
+      </c>
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>10:45</t>
+        </is>
+      </c>
+      <c r="E10" t="n">
+        <v>1.25</v>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>Track Block</t>
+        </is>
+      </c>
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
+          <t>B110</t>
+        </is>
+      </c>
+      <c r="B11" t="inlineStr">
+        <is>
+          <t>SEC-C</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="E11" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>Track Block</t>
+        </is>
+      </c>
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>B111</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>SEC-C</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="E12" t="n">
+        <v>2</v>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>Track Block</t>
+        </is>
+      </c>
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>B112</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>SEC-C</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>16:30</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="E13" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>OHE Block</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>B113</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
           <t>SEC-D</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="D14" t="inlineStr">
+        <is>
+          <t>13:30</t>
+        </is>
+      </c>
+      <c r="E14" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>Track Block</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>B114</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>SEC-D</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>12:30</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
         <is>
           <t>14:30</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>17:00</t>
-        </is>
-      </c>
-      <c r="E10" t="n">
+      <c r="E15" t="n">
+        <v>2</v>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>OHE Block</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>B115</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>SEC-D</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>14:45</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>17:15</t>
+        </is>
+      </c>
+      <c r="E16" t="n">
         <v>2.5</v>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F16" t="inlineStr">
         <is>
           <t>OHE Block</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr">
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>B116</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>SEC-E</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr">
+        <is>
+          <t>09:00</t>
+        </is>
+      </c>
+      <c r="D17" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="E17" t="n">
+        <v>2.5</v>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>Track Block</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>B117</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>SEC-F</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>12:00</t>
+        </is>
+      </c>
+      <c r="E18" t="n">
+        <v>2</v>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>Track Block</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>Available</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
+        <is>
+          <t>B118</t>
+        </is>
+      </c>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>SEC-G</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="D19" t="inlineStr">
+        <is>
+          <t>16:00</t>
+        </is>
+      </c>
+      <c r="E19" t="n">
+        <v>3</v>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>Track Block</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
         <is>
           <t>Available</t>
         </is>
@@ -1617,7 +3276,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F11"/>
+  <dimension ref="A1:F16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1655,7 +3314,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>A001</t>
+          <t>A101</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
@@ -1670,7 +3329,7 @@
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Warning</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -1687,7 +3346,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>A002</t>
+          <t>A102</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
@@ -1719,17 +3378,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>A003</t>
+          <t>A103</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>OHE</t>
+          <t>Track</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>SEC-B</t>
+          <t>SEC-A</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -1739,120 +3398,120 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>A004</t>
+          <t>A104</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>Track</t>
+          <t>OHE</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>SEC-C</t>
+          <t>SEC-A</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>A005</t>
+          <t>A105</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>Signal</t>
+          <t>Track</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>SEC-C</t>
+          <t>SEC-B</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Warning</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-15</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>A006</t>
+          <t>A106</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>OHE</t>
+          <t>Signal</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>SEC-A</t>
+          <t>SEC-B</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Good</t>
+          <t>Critical</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-16</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>A007</t>
+          <t>A107</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>Track</t>
+          <t>OHE</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
@@ -1867,24 +3526,24 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-18</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>A008</t>
+          <t>A108</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>Signal</t>
+          <t>Track</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
@@ -1894,34 +3553,34 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>Critical</t>
+          <t>Good</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-24</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-21</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>A009</t>
+          <t>A109</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>Bridge</t>
+          <t>Track</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>SEC-D</t>
+          <t>SEC-C</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -1931,44 +3590,204 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-17</t>
         </is>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>A010</t>
+          <t>A110</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
+          <t>Signal</t>
+        </is>
+      </c>
+      <c r="C11" t="inlineStr">
+        <is>
+          <t>SEC-C</t>
+        </is>
+      </c>
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
+        <is>
+          <t>2026-08-18</t>
+        </is>
+      </c>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>2026-09-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" t="inlineStr">
+        <is>
+          <t>A111</t>
+        </is>
+      </c>
+      <c r="B12" t="inlineStr">
+        <is>
+          <t>Track</t>
+        </is>
+      </c>
+      <c r="C12" t="inlineStr">
+        <is>
+          <t>SEC-C</t>
+        </is>
+      </c>
+      <c r="D12" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E12" t="inlineStr">
+        <is>
+          <t>2026-08-05</t>
+        </is>
+      </c>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>2026-09-16</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>A112</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
           <t>OHE</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr">
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>SEC-C</t>
+        </is>
+      </c>
+      <c r="D13" t="inlineStr">
+        <is>
+          <t>Warning</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>2026-08-16</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>2026-09-18</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>A113</t>
+        </is>
+      </c>
+      <c r="B14" t="inlineStr">
+        <is>
+          <t>Bridge</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
         <is>
           <t>SEC-D</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr">
+      <c r="D14" t="inlineStr">
         <is>
           <t>Critical</t>
         </is>
       </c>
-      <c r="E11" t="inlineStr">
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>2026-07-30</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>2026-09-20</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>A114</t>
+        </is>
+      </c>
+      <c r="B15" t="inlineStr">
+        <is>
+          <t>OHE</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>SEC-D</t>
+        </is>
+      </c>
+      <c r="D15" t="inlineStr">
+        <is>
+          <t>Critical</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
         <is>
           <t>2026-08-01</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr">
+      <c r="F15" t="inlineStr">
         <is>
           <t>2026-09-14</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>A115</t>
+        </is>
+      </c>
+      <c r="B16" t="inlineStr">
+        <is>
+          <t>Signal</t>
+        </is>
+      </c>
+      <c r="C16" t="inlineStr">
+        <is>
+          <t>SEC-D</t>
+        </is>
+      </c>
+      <c r="D16" t="inlineStr">
+        <is>
+          <t>Warning</t>
+        </is>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>2026-08-14</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>2026-09-19</t>
         </is>
       </c>
     </row>

</xml_diff>